<commit_message>
Docs and ReadMes: CT supplemental files are not read here
README and landing page: new section on what the repository does not read --
the CDISC CT Rules documents and Codetable Mapping files -- with public
references (CT page, 2023-06-22 webinar, IS Knowledge Base article).
SDTMIG_Statements and Immunogenicity_Findings ReadMe: the same note under
KNOWN GAPS. Codelist_Phrases ReadMe: an example of an NCIt synonym that names
one of two sibling terms (HLA in ISBDAGT). ReadMe sheets only; data sheets and
content hashes unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzUu6ftcm2k3S6ZiuqP
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTMIG_Statements.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTMIG_Statements.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A63"/>
+  <dimension ref="A1:A66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -695,179 +695,183 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>The IG refers to the CDISC CT Rules for some choices (e.g. IS-A7: when to use each of the two ISBDAGNT</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>SHEETS</t>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  codelists). The CT supplemental files -- Rules documents and Codetable Mapping files, listed on the</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Statements — one row per quoted statement.</t>
+          <t xml:space="preserve">  cdisc.org Controlled Terminology page -- are not read here. They may refine the statements quoted.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Variables — one row per variable in Variables_Named: the SDTMIG v3.4 variable-table row as published,</t>
-        </is>
-      </c>
+      <c r="A37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  plus Named_In. An empty CDISC CT Codelist Code(s) means the table gives no codelist (e.g. PCTESTCD).</t>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>SHEETS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Provenance — versions; per sheet rows, columns and a content hash.</t>
+          <t>Statements — one row per quoted statement.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Variables — one row per variable in Variables_Named: the SDTMIG v3.4 variable-table row as published,</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>COLUMNS — Statements</t>
+          <t xml:space="preserve">  plus Named_In. An empty CDISC CT Codelist Code(s) means the table gives no codelist (e.g. PCTESTCD).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Statement_ID: domain + A + assumption item (+ sub-item), e.g. IS-A7b; 4.1.9-n for the §4.1.9 passages in</t>
+          <t>Provenance — versions; per sheet rows, columns and a content hash.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  order; &lt;variable&gt;-Notes for CDISC Notes. RS-DR = RS Disease Response Use Case Assumptions;</t>
-        </is>
-      </c>
+      <c r="A43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  RS-CC = RS Clinical Classifications Use Case Assumptions.</t>
+          <t>COLUMNS — Statements</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Selected_As: facet | routing | record — why the row was selected.</t>
+          <t>Statement_ID: domain + A + assumption item (+ sub-item), e.g. IS-A7b; 4.1.9-n for the §4.1.9 passages in</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Source: the document and its date.</t>
+          <t xml:space="preserve">  order; &lt;variable&gt;-Notes for CDISC Notes. RS-DR = RS Disease Response Use Case Assumptions;</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Section: the numbered IG section; for Assumptions also the Assumptions heading.</t>
+          <t xml:space="preserve">  RS-CC = RS Clinical Classifications Use Case Assumptions.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Item: assumption item and lettered sub-item. An item row holds the item's text before its first sub-item;</t>
+          <t>Selected_As: facet | routing | record — why the row was selected.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  a sub-item row keeps its roman sub-items (e.g. 1c holds i-iv).</t>
+          <t>Source: the document and its date.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Page: page in the IG (printed page = PDF page). Empty for CDISC Notes (CSV).</t>
+          <t>Section: the numbered IG section; for Assumptions also the Assumptions heading.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Domain: the dataset whose Assumptions or Notes the text belongs to; empty for §4.1.9.</t>
+          <t>Item: assumption item and lettered sub-item. An item row holds the item's text before its first sub-item;</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Variables_Named: words that are variables of the dataset their first two letters name, in the SDTMIG v3.4</t>
+          <t xml:space="preserve">  a sub-item row keeps its roman sub-items (e.g. 1c holds i-iv).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  variable table; in order of first appearance.</t>
+          <t>Page: page in the IG (printed page = PDF page). Empty for CDISC Notes (CSV).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Model_Variables_Named: words not in that dataset's SDTMIG v3.4 table whose -- form is an SDTM v2.0 variable</t>
+          <t>Domain: the dataset whose Assumptions or Notes the text belongs to; empty for §4.1.9.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of the dataset's observation class (e.g. LBPOS and LBLOC in LB-A8: --POS and --LOC, Findings).</t>
+          <t>Variables_Named: words that are variables of the dataset their first two letters name, in the SDTMIG v3.4</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Domains_Named: dataset codes written as (XX) or "XX domain"; in order of first appearance.</t>
+          <t xml:space="preserve">  variable table; in order of first appearance.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Text: the statement, verbatim.</t>
+          <t>Model_Variables_Named: words not in that dataset's SDTMIG v3.4 table whose -- form is an SDTM v2.0 variable</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of the dataset's observation class (e.g. LBPOS and LBLOC in LB-A8: --POS and --LOC, Findings).</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>COLUMNS — Variables</t>
+          <t>Domains_Named: dataset codes written as (XX) or "XX domain"; in order of first appearance.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>The columns of SDTMIG_v3.4.csv, unchanged, plus Named_In: the Statement_IDs that name the variable.</t>
+          <t>Text: the statement, verbatim.</t>
         </is>
       </c>
     </row>
@@ -875,14 +879,31 @@
       <c r="A61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>READING</t>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>COLUMNS — Variables</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>The columns of SDTMIG_v3.4.csv, unchanged, plus Named_In: the Statement_IDs that name the variable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>READING</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Read with keep_default_na=False (pandas) or the equivalent, so that no cell is read as missing.</t>
         </is>

</xml_diff>